<commit_message>
docs: clarify UNICEF operator plan and simplify reply
Apply approved feedback without changing budgets, staffing shares or targets.
Clarify ASP control, exit eligibility, mobile gates and review assumptions.
</commit_message>
<xml_diff>
--- a/outputs/unicef-2026-09-10/Annex_C_Template_3_Galeon_PrivacyProtocol_2026-09.xlsx
+++ b/outputs/unicef-2026-09-10/Annex_C_Template_3_Galeon_PrivacyProtocol_2026-09.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Design and Data Plan" sheetId="1" r:id="R8e98ad9558b54766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Design and Data Plan" sheetId="1" r:id="R97bc610785654101"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1071,7 +1071,7 @@
 Fabio Anaya (ops) 5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="125" customHeight="1">
+    <x:row r="8" ht="140" customHeight="1">
       <x:c r="A8" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 1</x:t>
@@ -1084,7 +1084,7 @@
         <x:v>Preserve repeated receipts and practical withdrawals while selecting an affordable, reviewable implementation.</x:v>
       </x:c>
       <x:c r="D8" s="111" t="str">
-        <x:v>1 decision by day 30 compares batching, multiWithdraw, mergeDeposit and verified upstream alternatives; Base/native USDC preferred. Public source, setup provenance and review required for any adopted custom circuit; no development-key artifact in the reviewed release. No V2 capability assumed.</x:v>
+        <x:v>1 decision by day 30 compares batching, multiWithdraw, mergeDeposit and verified upstream alternatives; Base/native USDC preferred. Preserve repeated receipts and practical partial withdrawals; merging is an option, not a required custom circuit. Any adopted custom circuit needs public source, setup provenance and a costed, scheduled review route. No development-key artifact or assumed V2 capability.</x:v>
       </x:c>
       <x:c r="E8" s="111" t="str">
         <x:v>Public GitHub decision record, source/commit and setup references, reproducible feasibility runs and an updated risk register.</x:v>
@@ -1255,7 +1255,7 @@
 Fabio Anaya (ops) 17.5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="125" customHeight="1">
+    <x:row r="17" ht="140" customHeight="1">
       <x:c r="A17" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 2</x:t>
@@ -1268,7 +1268,7 @@
         <x:v>Create a measurable pipeline that can support real activity after review.</x:v>
       </x:c>
       <x:c r="D17" s="111" t="str">
-        <x:v>1 Q3 cohort plan of 20 places and 3 further Q4 cohorts of 20; 50% activation is an unvalidated assumption. Qualify independent channels, an integration candidate and external funding sources; distinguish interest, commitment and funds available. No forced lockup or grant-funded pool principal.</x:v>
+        <x:v>1 Q3 cohort plan of 20 places and 3 further Q4 cohorts of 20; 50% activation is unvalidated. Qualify independent channels, 1 integration candidate and external funding sources. Record amounts, ordinary payment needs, expected withdrawals and replenishment; distinguish interest, commitments and available funds. No forced lockup or grant-funded pool principal.</x:v>
       </x:c>
       <x:c r="E17" s="111" t="str">
         <x:v>Online recruitment/resource tracker with contacts, source, amount, availability and next step; public aggregate funnel updated weekly.</x:v>
@@ -1335,7 +1335,7 @@
 Fabio Anaya (ops) 17.5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="125" customHeight="1">
+    <x:row r="21" ht="140" customHeight="1">
       <x:c r="A21" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 2</x:t>
@@ -1348,7 +1348,7 @@
         <x:v>Test legal boundaries against the actual operator/key/data model and resource the funded year responsibly.</x:v>
       </x:c>
       <x:c r="D21" s="111" t="str">
-        <x:v>1 counsel memo for Colombia or selected pilot jurisdiction; 1 responsibility matrix and legal-risk register. Non-custody is not assumed to remove obligations. Scope ASP policy/terms, data/reporting ownership and specialist review procurement; no licence or off-ramp acceptance claimed in advance.</x:v>
+        <x:v>1 counsel memo for Colombia or selected pilot jurisdiction; 1 responsibility matrix and legal-risk register. Assess Cartagena On Chain as proposed initial ASP operator for the capped trial, separately from relayer and partner programme roles. Scope actual powers, policy/terms, data/reporting and review procurement. Non-custody alone does not establish permission; no licence or off-ramp acceptance assumed.</x:v>
       </x:c>
       <x:c r="E21" s="111" t="str">
         <x:v>Counsel scope and findings in controlled online evidence folder; dated procurement, administration and quarterly-reporting trackers.</x:v>
@@ -1659,7 +1659,7 @@
 Fabio Anaya (ops) 15%</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="125" customHeight="1">
+    <x:row r="40" ht="140" customHeight="1">
       <x:c r="A40" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 1</x:t>
@@ -1672,7 +1672,7 @@
         <x:v>An accepting operator can control the canonical policy/root without hidden founder overrides.</x:v>
       </x:c>
       <x:c r="D40" s="111" t="str">
-        <x:v>≥15 ASP scenarios cover decisions, manual add/remove with reason/audit trail, restart/root rebuild, outage, stale roots, rotation, backups and exits. Separate ASP/relayer credentials. ≥8 governance tests cover verifier, upgrade, fee, registry and role bypasses; proposed 48-hour delay, routine roots separately controlled.</x:v>
+        <x:v>≥15 ASP scenarios cover acceptance/rejection of association-set inclusion, manual correction with reasons/audit trail, decisions preserved after restart/root rebuild, outage, stale roots, rotation, backups and eligible-depositor exits. Separate ASP/relayer credentials. ≥8 governance tests cover verifier, upgrade, fee, registry and role bypasses; proposed 48-hour delay, routine roots separately controlled.</x:v>
       </x:c>
       <x:c r="E40" s="111" t="str">
         <x:v>Public self-hosting runbook, policy/root manifests and CI scenarios; key-role evidence with secrets redacted. Reviewer findings tracked to closure.</x:v>
@@ -2103,7 +2103,7 @@
 Fabio Anaya (ops) 2.5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="125" customHeight="1">
+    <x:row r="64" ht="150" customHeight="1">
       <x:c r="A64" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 2</x:t>
@@ -2116,7 +2116,7 @@
         <x:v>Generate observable real activity without claiming a production aid-delivery service.</x:v>
       </x:c>
       <x:c r="D64" s="111" t="str">
-        <x:v>1 integration live by mid-month 9; ≥14 days observed before Q3 end. Publish reviewed caps, role holders, monitoring and incident stops. Required authority restrictions, tested exits and physical-device acceptance precede external use. If missed, report the miss and request an amendment; no automatic pass.</x:v>
+        <x:v>1 integration live by mid-month 9; ≥14 days observed before Q3 end. Cartagena On Chain is the proposed initial ASP operator, including if no independent alternative joins, subject to Q1 legal/role assessment and release checks. Publish caps, actual ASP/relayer role holders, monitoring and incident stops. Authority restrictions, eligible-depositor exits and Android gates precede use. A missed gate/date requires a reported miss and proposed amendment.</x:v>
       </x:c>
       <x:c r="E64" s="111" t="str">
         <x:v>Public deployment and aggregate uptime/flow dashboard; controlled signed operator/resource checklist, legal update and incident runbook.</x:v>
@@ -2159,7 +2159,7 @@
 Fabio Anaya (ops) 15%</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="125" customHeight="1">
+    <x:row r="67" ht="140" customHeight="1">
       <x:c r="A67" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 1</x:t>
@@ -2172,7 +2172,7 @@
         <x:v>The reference PWA works safely on the devices users will actually carry.</x:v>
       </x:c>
       <x:c r="D67" s="111" t="str">
-        <x:v>On 2 physical Android models (3 GB / 4 GB): ≥30 attempts each, warm-cache proving p95 ≤60 s and ≥95% proof completion, failures included. Complete wallet handoff, restart/network-loss, low-memory, concurrent-root and lost/shared-phone tests in months 7–8; report cold download and end-to-end time separately.</x:v>
+        <x:v>On 2 physical Android models (3 GB / 4 GB): ≥30 attempts each, warm-cache proof-generation p95 ≤60 s and ≥95% proof-generation completion, failures included. Pass Q1 network/cold-start thresholds, wallet handoff, restart/network-loss, low-memory, concurrent-root and lost/shared-phone tests in months 7–8 before external use. Record cold downloads and end-to-end time separately.</x:v>
       </x:c>
       <x:c r="E67" s="111" t="str">
         <x:v>Device/version and benchmark dataset, timing distribution, failure traces and anonymized task evidence; release-gate checklist and relevant re-review records.</x:v>
@@ -2183,7 +2183,7 @@
 Fabio Anaya (ops) 7.5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="125" customHeight="1">
+    <x:row r="68" ht="140" customHeight="1">
       <x:c r="A68" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 2</x:t>
@@ -2196,7 +2196,7 @@
         <x:v>Show tested exits and revocation of superseded powers without overstating decentralisation.</x:v>
       </x:c>
       <x:c r="D68" s="111" t="str">
-        <x:v>1 handover/rotation with old powers revoked; persistent manual correction/root rebuild verified. Reference UI supports eligible depositor ragequit and direct submission during relayer outage, with gas/privacy warnings. ≥10 successful alternate-relayer submissions with primary disabled. Target 1 independently controlled operator; if unmet, report that target missed, separately from team-controlled failover.</x:v>
+        <x:v>1 handover/rotation with old powers revoked; persistent correction/root rebuild verified. Reference UI tests exits for eligible original depositors with valid note proof, plus direct withdrawal during relayer outage; disclose eligibility, gas and privacy limits. ≥10 successful alternate-relayer submissions with primary disabled. Target 1 independent relayer operator; team-run failover does not meet independence. If recruitment fails, report that target missed.</x:v>
       </x:c>
       <x:c r="E68" s="111" t="str">
         <x:v>Public runbooks and redacted role/transaction evidence; controlled operator outreach/acceptance tracker distinguishes team-operated instances from independent operation.</x:v>
@@ -2571,7 +2571,7 @@
 Fabio Anaya (ops) 5%</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" ht="125" customHeight="1">
+    <x:row r="89" ht="140" customHeight="1">
       <x:c r="A89" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 1</x:t>
@@ -2584,7 +2584,7 @@
         <x:v>Preserve reliable mobile and provenance behavior as fixes are integrated.</x:v>
       </x:c>
       <x:c r="D89" s="111" t="str">
-        <x:v>1 versioned release passes the ≥12 disclosure fixtures and the 2-device Android gate (≥30 attempts/device, p95 ≤60 s warm-cache proving, ≥95% completion). Rerun secret-storage, no-duplicate/no-false-paid recovery and supported multipayment flows.</x:v>
+        <x:v>1 versioned release passes ≥12 disclosure fixtures and the 2-device Android gate: ≥30 attempts/device, warm-cache proof-generation p95 ≤60 s, ≥95% proof-generation completion and the Q1 network/cold-start thresholds. Rerun secret-storage, no-duplicate/no-false-paid recovery and supported multipayment flows.</x:v>
       </x:c>
       <x:c r="E89" s="111" t="str">
         <x:v>Public release artifacts, reproducible CI/benchmark results and change/provenance manifest; controlled consent-based regression evidence.</x:v>
@@ -2755,7 +2755,7 @@
 Fabio Anaya (ops) 20%</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="125" customHeight="1">
+    <x:row r="98" ht="140" customHeight="1">
       <x:c r="A98" s="89" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Activity 2</x:t>
@@ -2768,7 +2768,7 @@
         <x:v>Test whether genuine external resources remain available; inflows alone do not establish retained balance.</x:v>
       </x:c>
       <x:c r="D98" s="111" t="str">
-        <x:v>≥USD 5,000 median externally sourced active balance over the final 30 consecutive days; 30 daily observations required. EXTERNAL RESOURCES REQUIRED: principal is not grant-funded or secured. Apply Q1 attribution/unknown-source method; assess withdrawals and replenishment. No forced lockup, yield promise or inference from USD 10,000 inflows.</x:v>
+        <x:v>≥USD 5,000 median externally sourced active balance over the final 30 consecutive days; 30 daily observations. EXTERNAL RESOURCES REQUIRED: principal is not grant-funded or secured. Test the Q1 resource plan: opening balances, ordinary payment needs, withdrawal timing and genuine replenishment. Apply the attribution/unknown-source method. No forced lockup, yield promise or inference from USD 10,000 cumulative inflows.</x:v>
       </x:c>
       <x:c r="E98" s="111" t="str">
         <x:v>Public daily-balance series, full-window median calculation and attribution methodology; controlled resource/availability evidence. Report any shortfall as a missed target.</x:v>
@@ -3091,20 +3091,20 @@
       <x:c r="E119" s="105" t="n"/>
       <x:c r="F119" s="105" t="n"/>
     </x:row>
-    <x:row r="120" ht="53" customHeight="1">
+    <x:row r="120" ht="60" customHeight="1">
       <x:c r="A120" s="105" t="n"/>
       <x:c r="B120" s="107" t="str">
-        <x:v>Operator control: Q2 self-hosted ASP/handover core, persistent manual correction, separately controlled roots/relayers and timelocked privileged changes; Q3 replacement/failover. Reference UI includes eligible depositor exit and direct submission. Automated screening adapters and formal appeal case-management are outside the baseline.</x:v>
+        <x:v>ASP: documented acceptance/rejection and persistent corrections; Q2 self-hosting, handover, controlled roots and timelocked privileges. Cartagena is the proposed initial ASP operator, subject to legal/role and release checks. Q3 tests replacement and relayer failover; independent relayer recruitment is a separate target. Exits require eligible original-depositor proof. Automated screening and formal appeals are outside scope.</x:v>
       </x:c>
       <x:c r="C120" s="105" t="n"/>
       <x:c r="D120" s="105" t="n"/>
       <x:c r="E120" s="105" t="n"/>
       <x:c r="F120" s="105" t="n"/>
     </x:row>
-    <x:row r="121" ht="53" customHeight="1">
+    <x:row r="121" ht="60" customHeight="1">
       <x:c r="A121" s="105" t="n"/>
       <x:c r="B121" s="107" t="str">
-        <x:v>One Android-capable PWA, not a native app. Before external use: two physical 3/4-GB devices, ≥30 attempts each, warm-cache proof p95 ≤60 s and ≥95% completion; protected secrets, wallet handoff and recovery gates. A second-EVM full-stack test completes in Q4; no second production pool.</x:v>
+        <x:v>One Android-capable PWA, not a native app. Before external use: two physical 3/4-GB devices, ≥30 attempts each, warm-cache proof-generation p95 ≤60 s, ≥95% proof-generation completion and Q1 network/cold-start thresholds; protected secrets, wallet handoff and recovery gates. Repeat in Q4. A second-EVM full-stack test completes in Q4; no second production pool.</x:v>
       </x:c>
       <x:c r="C121" s="105" t="n"/>
       <x:c r="D121" s="105" t="n"/>
@@ -3143,10 +3143,10 @@
       <x:c r="E124" s="105" t="n"/>
       <x:c r="F124" s="105" t="n"/>
     </x:row>
-    <x:row r="125" ht="53" customHeight="1">
+    <x:row r="125" ht="60" customHeight="1">
       <x:c r="A125" s="105" t="n"/>
       <x:c r="B125" s="107" t="str">
-        <x:v>Day-30 decision preserves practical multipayment UX while choosing a sourced, affordable path. No development-key circuit in the reviewed release; any adopted custom circuit requires public source, documented ceremony/setup provenance and costed independent review. Do not assume upstream V2 capabilities.</x:v>
+        <x:v>Day-30 decision preserves repeated receipts and practical partial withdrawals; merging is an architecture option, not an automatic custom-circuit commitment. No development-key artifact in the reviewed release. Any custom circuit needs public source, ceremony/setup provenance and an affordable, scheduled independent review route. No upstream V2 capability assumed.</x:v>
       </x:c>
       <x:c r="C125" s="105" t="n"/>
       <x:c r="D125" s="105" t="n"/>
@@ -9457,6 +9457,6 @@
     <x:mergeCell ref="B131:F131"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R314bb2f760f24276"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf82eb3141e4454"/>
 </x:worksheet>
 </file>
</xml_diff>